<commit_message>
cleaned the '01_input_prepared' directory
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://studentcbs-my.sharepoint.com/personal/djh_eco_cbs_dk/Documents/Documents/GitHub/Nord_H2ub/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\ammonia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{3CB9F67F-4C4D-45E8-9CB3-A251766F4AB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5E111EC9-FCB4-4C2A-9F74-479F2DAF01E9}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7D5FC6-FA31-40DD-AEA0-3F277DDD5CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-11730" yWindow="-21720" windowWidth="51840" windowHeight="21240" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="4" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="123">
   <si>
     <t>Unit</t>
   </si>
@@ -416,6 +416,33 @@
   </si>
   <si>
     <t>24h</t>
+  </si>
+  <si>
+    <t>solar_plant_node</t>
+  </si>
+  <si>
+    <t>wind_onshore_plant_node</t>
+  </si>
+  <si>
+    <t>wind_offshore_plant_node</t>
+  </si>
+  <si>
+    <t>pl_wholesale_solar</t>
+  </si>
+  <si>
+    <t>pl_solar_PPA</t>
+  </si>
+  <si>
+    <t>pl_wholesale_wind_onshore</t>
+  </si>
+  <si>
+    <t>pl_wind_onshore_PPA</t>
+  </si>
+  <si>
+    <t>pl_wholesale_wind_offshore</t>
+  </si>
+  <si>
+    <t>pl_wind_offshore_PPA</t>
   </si>
 </sst>
 </file>
@@ -519,7 +546,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -535,6 +562,8 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1346,8 +1375,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{856854C3-DC05-4AB8-91B8-0E52D9C11DBC}" name="Table13" displayName="Table13" ref="A1:AA5" totalsRowShown="0">
-  <autoFilter ref="A1:AA5" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{856854C3-DC05-4AB8-91B8-0E52D9C11DBC}" name="Table13" displayName="Table13" ref="A1:AA11" totalsRowShown="0">
+  <autoFilter ref="A1:AA11" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
   <tableColumns count="27">
     <tableColumn id="1" xr3:uid="{26B0CA71-1EA9-44CF-8E6D-31054ECA99A6}" name="Connection"/>
     <tableColumn id="26" xr3:uid="{E67F4435-EF76-417C-B715-53719E5FB41F}" name="Object_type"/>
@@ -1711,23 +1740,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576C757C-091A-46DF-949E-B17661031FDE}">
   <dimension ref="A1:R12"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.81640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.81640625" customWidth="1"/>
-    <col min="3" max="3" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.36328125" customWidth="1"/>
-    <col min="5" max="5" width="16.7265625" bestFit="1" customWidth="1"/>
-    <col min="6" max="12" width="10.54296875" customWidth="1"/>
-    <col min="13" max="13" width="12.7265625" customWidth="1"/>
+    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.85546875" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="12" width="10.5703125" customWidth="1"/>
+    <col min="13" max="13" width="12.7109375" customWidth="1"/>
     <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.26953125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.1796875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1783,7 +1812,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" s="9" t="s">
         <v>66</v>
       </c>
@@ -1791,12 +1820,12 @@
         <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>114</v>
       </c>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>93</v>
       </c>
@@ -1804,12 +1833,12 @@
         <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>115</v>
       </c>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
         <v>94</v>
       </c>
@@ -1817,12 +1846,12 @@
         <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>116</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
         <v>76</v>
       </c>
@@ -1844,7 +1873,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
         <v>101</v>
       </c>
@@ -1860,7 +1889,7 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
         <v>104</v>
       </c>
@@ -1891,7 +1920,7 @@
       <c r="P7" s="1"/>
       <c r="Q7" s="2"/>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>99</v>
       </c>
@@ -1904,18 +1933,18 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="9"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
     </row>
@@ -1949,14 +1978,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CABA7C5-6230-4207-9D35-0A95D86E66AC}">
   <dimension ref="A1:Q10"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6328125" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" customWidth="1"/>
-    <col min="7" max="8" width="9.81640625" customWidth="1"/>
+    <col min="1" max="1" width="14.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="7" max="8" width="9.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2009,7 +2038,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>66</v>
       </c>
@@ -2020,8 +2049,8 @@
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
-      <c r="G2" s="3" t="s">
-        <v>67</v>
+      <c r="G2" t="s">
+        <v>114</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="7"/>
@@ -2034,7 +2063,7 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>93</v>
       </c>
@@ -2045,8 +2074,8 @@
       <c r="D3" s="4"/>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
-      <c r="G3" s="4" t="s">
-        <v>67</v>
+      <c r="G3" t="s">
+        <v>115</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -2059,7 +2088,7 @@
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>94</v>
       </c>
@@ -2070,8 +2099,8 @@
       <c r="D4" s="3"/>
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
-      <c r="G4" s="3" t="s">
-        <v>67</v>
+      <c r="G4" t="s">
+        <v>116</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -2084,7 +2113,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>76</v>
       </c>
@@ -2119,7 +2148,7 @@
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>101</v>
       </c>
@@ -2152,7 +2181,7 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>104</v>
       </c>
@@ -2197,7 +2226,7 @@
       </c>
       <c r="Q7" s="4"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>99</v>
       </c>
@@ -2226,7 +2255,7 @@
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -2268,34 +2297,34 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C870BDA0-9E4C-481D-87BE-9D47789809C8}">
-  <dimension ref="A1:AA5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:AA11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.36328125" customWidth="1"/>
-    <col min="2" max="2" width="19.54296875" customWidth="1"/>
-    <col min="3" max="6" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.26953125" customWidth="1"/>
-    <col min="9" max="9" width="17.453125" customWidth="1"/>
-    <col min="10" max="10" width="15.453125" customWidth="1"/>
-    <col min="11" max="11" width="17.453125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.453125" customWidth="1"/>
+    <col min="1" max="1" width="15.42578125" customWidth="1"/>
+    <col min="2" max="2" width="19.5703125" customWidth="1"/>
+    <col min="3" max="6" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="17.42578125" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" customWidth="1"/>
+    <col min="11" max="11" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.42578125" customWidth="1"/>
     <col min="13" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="15.453125" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" customWidth="1"/>
     <col min="15" max="15" width="19" customWidth="1"/>
-    <col min="16" max="16" width="10.54296875" customWidth="1"/>
-    <col min="17" max="17" width="15.54296875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.1796875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.81640625" customWidth="1"/>
-    <col min="21" max="21" width="12.81640625" customWidth="1"/>
-    <col min="22" max="23" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="35.26953125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.5703125" customWidth="1"/>
+    <col min="17" max="17" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.140625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.85546875" customWidth="1"/>
+    <col min="21" max="21" width="12.85546875" customWidth="1"/>
+    <col min="22" max="23" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -2378,7 +2407,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -2437,7 +2466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>75</v>
       </c>
@@ -2493,7 +2522,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>109</v>
       </c>
@@ -2519,7 +2548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -2554,6 +2583,297 @@
         <v>55</v>
       </c>
       <c r="AA5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>117</v>
+      </c>
+      <c r="B6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D6" t="s">
+        <v>114</v>
+      </c>
+      <c r="E6" t="s">
+        <v>114</v>
+      </c>
+      <c r="F6" t="s">
+        <v>69</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H6">
+        <v>1000</v>
+      </c>
+      <c r="I6">
+        <v>1000</v>
+      </c>
+      <c r="J6">
+        <v>1000</v>
+      </c>
+      <c r="K6">
+        <v>1000</v>
+      </c>
+      <c r="L6">
+        <v>1000</v>
+      </c>
+      <c r="M6">
+        <v>1000</v>
+      </c>
+      <c r="N6">
+        <v>1000</v>
+      </c>
+      <c r="O6">
+        <v>1000</v>
+      </c>
+      <c r="R6">
+        <v>1</v>
+      </c>
+      <c r="T6">
+        <v>1</v>
+      </c>
+      <c r="Z6" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>118</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" t="s">
+        <v>114</v>
+      </c>
+      <c r="E7" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H7">
+        <v>1000</v>
+      </c>
+      <c r="I7">
+        <v>1000</v>
+      </c>
+      <c r="L7">
+        <v>1000</v>
+      </c>
+      <c r="M7">
+        <v>1000</v>
+      </c>
+      <c r="T7">
+        <v>1</v>
+      </c>
+      <c r="Z7" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>119</v>
+      </c>
+      <c r="B8" t="s">
+        <v>51</v>
+      </c>
+      <c r="C8" t="s">
+        <v>69</v>
+      </c>
+      <c r="D8" t="s">
+        <v>115</v>
+      </c>
+      <c r="E8" t="s">
+        <v>115</v>
+      </c>
+      <c r="F8" t="s">
+        <v>69</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H8">
+        <v>1000</v>
+      </c>
+      <c r="I8">
+        <v>1000</v>
+      </c>
+      <c r="J8">
+        <v>1000</v>
+      </c>
+      <c r="K8">
+        <v>1000</v>
+      </c>
+      <c r="L8">
+        <v>1000</v>
+      </c>
+      <c r="M8">
+        <v>1000</v>
+      </c>
+      <c r="N8">
+        <v>1000</v>
+      </c>
+      <c r="O8">
+        <v>1000</v>
+      </c>
+      <c r="R8">
+        <v>1</v>
+      </c>
+      <c r="T8">
+        <v>1</v>
+      </c>
+      <c r="Z8" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>120</v>
+      </c>
+      <c r="B9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>115</v>
+      </c>
+      <c r="E9" t="s">
+        <v>67</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H9">
+        <v>1000</v>
+      </c>
+      <c r="I9">
+        <v>1000</v>
+      </c>
+      <c r="L9">
+        <v>1000</v>
+      </c>
+      <c r="M9">
+        <v>1000</v>
+      </c>
+      <c r="T9">
+        <v>1</v>
+      </c>
+      <c r="Z9" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>121</v>
+      </c>
+      <c r="B10" t="s">
+        <v>51</v>
+      </c>
+      <c r="C10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" t="s">
+        <v>116</v>
+      </c>
+      <c r="E10" t="s">
+        <v>116</v>
+      </c>
+      <c r="F10" t="s">
+        <v>69</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H10">
+        <v>1000</v>
+      </c>
+      <c r="I10">
+        <v>1000</v>
+      </c>
+      <c r="J10">
+        <v>1000</v>
+      </c>
+      <c r="K10">
+        <v>1000</v>
+      </c>
+      <c r="L10">
+        <v>1000</v>
+      </c>
+      <c r="M10">
+        <v>1000</v>
+      </c>
+      <c r="N10">
+        <v>1000</v>
+      </c>
+      <c r="O10">
+        <v>1000</v>
+      </c>
+      <c r="R10">
+        <v>1</v>
+      </c>
+      <c r="T10">
+        <v>1</v>
+      </c>
+      <c r="Z10" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>122</v>
+      </c>
+      <c r="B11" t="s">
+        <v>51</v>
+      </c>
+      <c r="C11" t="s">
+        <v>116</v>
+      </c>
+      <c r="E11" t="s">
+        <v>67</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>32</v>
+      </c>
+      <c r="H11">
+        <v>1000</v>
+      </c>
+      <c r="I11">
+        <v>1000</v>
+      </c>
+      <c r="L11">
+        <v>1000</v>
+      </c>
+      <c r="M11">
+        <v>1000</v>
+      </c>
+      <c r="T11">
+        <v>1</v>
+      </c>
+      <c r="Z11" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="AA11">
         <v>1</v>
       </c>
     </row>
@@ -2582,22 +2902,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{981CFA5E-60F3-446F-A856-2FA65B76879A}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.1796875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.54296875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.54296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.81640625" customWidth="1"/>
-    <col min="8" max="8" width="12.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.85546875" customWidth="1"/>
+    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.26953125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.1796875" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -2632,7 +2952,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>74</v>
       </c>
@@ -2658,7 +2978,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>110</v>
       </c>
@@ -2707,117 +3027,117 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DC79B9-9C58-497E-9FD8-D3F2239E9BDC}">
   <dimension ref="A1:A22"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>108</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>111</v>
       </c>

</xml_diff>

<commit_message>
adjusted source files to match the current district heating mechanics
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\ammonia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF7D5FC6-FA31-40DD-AEA0-3F277DDD5CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF52CFD9-8946-4A9E-9C5F-5C0310861725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25695" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="4" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="123">
   <si>
     <t>Unit</t>
   </si>
@@ -310,12 +310,6 @@
     <t>initial_units_on</t>
   </si>
   <si>
-    <t>heat_low</t>
-  </si>
-  <si>
-    <t>heat_high</t>
-  </si>
-  <si>
     <t>Auxilliary</t>
   </si>
   <si>
@@ -443,13 +437,19 @@
   </si>
   <si>
     <t>pl_wind_offshore_PPA</t>
+  </si>
+  <si>
+    <t>excess_heat</t>
+  </si>
+  <si>
+    <t>heat</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -467,6 +467,13 @@
       <b/>
       <sz val="11"/>
       <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -546,7 +553,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -562,8 +569,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1742,18 +1748,24 @@
   <dimension ref="A1:R12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.85546875" customWidth="1"/>
-    <col min="3" max="3" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" customWidth="1"/>
-    <col min="5" max="5" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="12" width="10.5703125" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" customWidth="1"/>
-    <col min="14" max="14" width="11" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.28515625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.140625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:18" x14ac:dyDescent="0.25">
@@ -1764,7 +1776,7 @@
         <v>42</v>
       </c>
       <c r="C1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
@@ -1773,16 +1785,16 @@
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="G1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="H1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="I1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="J1" t="s">
         <v>61</v>
@@ -1820,33 +1832,33 @@
         <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B3" t="s">
         <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
         <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
@@ -1875,13 +1887,13 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B6" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="O6">
         <v>0.4</v>
@@ -1891,16 +1903,16 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B7" t="s">
+        <v>101</v>
+      </c>
+      <c r="C7" t="s">
         <v>104</v>
       </c>
-      <c r="B7" t="s">
-        <v>103</v>
-      </c>
-      <c r="C7" t="s">
-        <v>106</v>
-      </c>
       <c r="E7" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F7">
         <v>0.5</v>
@@ -1922,10 +1934,10 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B8" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C8" t="s">
         <v>72</v>
@@ -1980,9 +1992,16 @@
   <dimension ref="A1:Q10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
-    <col min="7" max="8" width="9.85546875" customWidth="1"/>
+    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="6" width="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="21.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.25">
@@ -1999,10 +2018,10 @@
         <v>2</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>3</v>
@@ -2011,31 +2030,31 @@
         <v>4</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>88</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>89</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.25">
@@ -2050,7 +2069,7 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="7"/>
@@ -2065,7 +2084,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>59</v>
@@ -2075,7 +2094,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -2090,7 +2109,7 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B4" t="s">
         <v>60</v>
@@ -2100,7 +2119,7 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -2132,7 +2151,7 @@
         <v>73</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>78</v>
+        <v>121</v>
       </c>
       <c r="I5" s="4"/>
       <c r="J5" s="4"/>
@@ -2150,10 +2169,10 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>67</v>
@@ -2162,10 +2181,10 @@
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
@@ -2183,10 +2202,10 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>73</v>
@@ -2195,18 +2214,16 @@
         <v>67</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>78</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7">
         <v>17.867924528301888</v>
@@ -2218,7 +2235,7 @@
       <c r="N7">
         <v>1.1506682867557716</v>
       </c>
-      <c r="O7" s="4">
+      <c r="O7" s="11">
         <v>7.6203703703703694</v>
       </c>
       <c r="P7" s="4">
@@ -2228,13 +2245,13 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
@@ -2300,18 +2317,19 @@
   <dimension ref="A1:AA11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.42578125" customWidth="1"/>
-    <col min="2" max="2" width="19.5703125" customWidth="1"/>
-    <col min="3" max="6" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.140625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.28515625" customWidth="1"/>
-    <col min="9" max="9" width="17.42578125" customWidth="1"/>
-    <col min="10" max="10" width="15.42578125" customWidth="1"/>
-    <col min="11" max="11" width="17.42578125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.42578125" customWidth="1"/>
-    <col min="13" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="15.42578125" customWidth="1"/>
-    <col min="15" max="15" width="19" customWidth="1"/>
+    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.140625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.85546875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10.5703125" customWidth="1"/>
     <col min="17" max="17" width="15.5703125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="17.140625" bestFit="1" customWidth="1"/>
@@ -2524,22 +2542,22 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="D4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F4" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G4" t="s">
         <v>32</v>
@@ -2556,7 +2574,7 @@
         <v>52</v>
       </c>
       <c r="C5" t="s">
-        <v>78</v>
+        <v>122</v>
       </c>
       <c r="E5" t="s">
         <v>71</v>
@@ -2588,7 +2606,7 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
         <v>51</v>
@@ -2597,15 +2615,15 @@
         <v>69</v>
       </c>
       <c r="D6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E6" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F6" t="s">
         <v>69</v>
       </c>
-      <c r="G6" s="11" t="s">
+      <c r="G6" t="s">
         <v>32</v>
       </c>
       <c r="H6">
@@ -2638,7 +2656,7 @@
       <c r="T6">
         <v>1</v>
       </c>
-      <c r="Z6" s="12" t="s">
+      <c r="Z6" t="s">
         <v>55</v>
       </c>
       <c r="AA6">
@@ -2647,18 +2665,18 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s">
         <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E7" t="s">
         <v>67</v>
       </c>
-      <c r="G7" s="11" t="s">
+      <c r="G7" t="s">
         <v>32</v>
       </c>
       <c r="H7">
@@ -2676,7 +2694,7 @@
       <c r="T7">
         <v>1</v>
       </c>
-      <c r="Z7" s="12" t="s">
+      <c r="Z7" t="s">
         <v>55</v>
       </c>
       <c r="AA7">
@@ -2685,7 +2703,7 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B8" t="s">
         <v>51</v>
@@ -2694,15 +2712,15 @@
         <v>69</v>
       </c>
       <c r="D8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E8" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F8" t="s">
         <v>69</v>
       </c>
-      <c r="G8" s="11" t="s">
+      <c r="G8" t="s">
         <v>32</v>
       </c>
       <c r="H8">
@@ -2735,7 +2753,7 @@
       <c r="T8">
         <v>1</v>
       </c>
-      <c r="Z8" s="12" t="s">
+      <c r="Z8" t="s">
         <v>55</v>
       </c>
       <c r="AA8">
@@ -2744,18 +2762,18 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B9" t="s">
         <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="E9" t="s">
         <v>67</v>
       </c>
-      <c r="G9" s="11" t="s">
+      <c r="G9" t="s">
         <v>32</v>
       </c>
       <c r="H9">
@@ -2773,7 +2791,7 @@
       <c r="T9">
         <v>1</v>
       </c>
-      <c r="Z9" s="12" t="s">
+      <c r="Z9" t="s">
         <v>55</v>
       </c>
       <c r="AA9">
@@ -2782,7 +2800,7 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="B10" t="s">
         <v>51</v>
@@ -2791,15 +2809,15 @@
         <v>69</v>
       </c>
       <c r="D10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E10" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F10" t="s">
         <v>69</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" t="s">
         <v>32</v>
       </c>
       <c r="H10">
@@ -2832,7 +2850,7 @@
       <c r="T10">
         <v>1</v>
       </c>
-      <c r="Z10" s="12" t="s">
+      <c r="Z10" t="s">
         <v>55</v>
       </c>
       <c r="AA10">
@@ -2841,18 +2859,18 @@
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="B11" t="s">
         <v>51</v>
       </c>
       <c r="C11" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E11" t="s">
         <v>67</v>
       </c>
-      <c r="G11" s="11" t="s">
+      <c r="G11" t="s">
         <v>32</v>
       </c>
       <c r="H11">
@@ -2870,7 +2888,7 @@
       <c r="T11">
         <v>1</v>
       </c>
-      <c r="Z11" s="12" t="s">
+      <c r="Z11" t="s">
         <v>55</v>
       </c>
       <c r="AA11">
@@ -2980,10 +2998,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -3074,7 +3092,7 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
@@ -3104,7 +3122,7 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
@@ -3124,22 +3142,22 @@
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
minor changes and bug fix
some comments where to change things to integrate further functionalities.
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\ammonia\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\ammonia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF52CFD9-8946-4A9E-9C5F-5C0310861725}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D1B9E0-7B43-446D-9025-82534FC356E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="124">
   <si>
     <t>Unit</t>
   </si>
@@ -443,6 +443,9 @@
   </si>
   <si>
     <t>heat</t>
+  </si>
+  <si>
+    <t>D</t>
   </si>
 </sst>
 </file>
@@ -1746,29 +1749,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576C757C-091A-46DF-949E-B17661031FDE}">
   <dimension ref="A1:R12"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.140625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.6640625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1824,7 +1827,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" s="9" t="s">
         <v>66</v>
       </c>
@@ -1837,7 +1840,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
         <v>91</v>
       </c>
@@ -1850,7 +1853,7 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
         <v>92</v>
       </c>
@@ -1863,7 +1866,7 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
         <v>76</v>
       </c>
@@ -1885,7 +1888,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
         <v>99</v>
       </c>
@@ -1901,7 +1904,7 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
         <v>102</v>
       </c>
@@ -1929,10 +1932,14 @@
       <c r="O7">
         <v>0.2</v>
       </c>
-      <c r="P7" s="1"/>
-      <c r="Q7" s="2"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="P7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
         <v>97</v>
       </c>
@@ -1945,18 +1952,18 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="10"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" s="9"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
     </row>
@@ -1990,21 +1997,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CABA7C5-6230-4207-9D35-0A95D86E66AC}">
   <dimension ref="A1:Q10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.85546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="21.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2057,7 +2064,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>66</v>
       </c>
@@ -2082,7 +2089,7 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
         <v>91</v>
       </c>
@@ -2107,7 +2114,7 @@
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>92</v>
       </c>
@@ -2132,7 +2139,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
         <v>76</v>
       </c>
@@ -2167,7 +2174,7 @@
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>99</v>
       </c>
@@ -2200,7 +2207,7 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>102</v>
       </c>
@@ -2243,7 +2250,7 @@
       </c>
       <c r="Q7" s="4"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
         <v>97</v>
       </c>
@@ -2272,7 +2279,7 @@
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="6"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6"/>
@@ -2315,34 +2322,34 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C870BDA0-9E4C-481D-87BE-9D47789809C8}">
   <dimension ref="A1:AA11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="25.6640625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.140625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.85546875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.5703125" customWidth="1"/>
-    <col min="17" max="17" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.85546875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.85546875" customWidth="1"/>
-    <col min="21" max="21" width="12.85546875" customWidth="1"/>
-    <col min="22" max="23" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="19.42578125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="35.28515625" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.109375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.5546875" customWidth="1"/>
+    <col min="17" max="17" width="15.5546875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.109375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.88671875" customWidth="1"/>
+    <col min="21" max="21" width="12.88671875" customWidth="1"/>
+    <col min="22" max="23" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="35.33203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -2425,7 +2432,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -2484,7 +2491,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>75</v>
       </c>
@@ -2540,7 +2547,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>107</v>
       </c>
@@ -2566,7 +2573,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>70</v>
       </c>
@@ -2604,7 +2611,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>115</v>
       </c>
@@ -2663,7 +2670,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>116</v>
       </c>
@@ -2701,7 +2708,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>117</v>
       </c>
@@ -2760,7 +2767,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>118</v>
       </c>
@@ -2798,7 +2805,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>119</v>
       </c>
@@ -2857,7 +2864,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>120</v>
       </c>
@@ -2920,22 +2927,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{981CFA5E-60F3-446F-A856-2FA65B76879A}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.85546875" customWidth="1"/>
-    <col min="8" max="8" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.88671875" customWidth="1"/>
+    <col min="8" max="8" width="12.88671875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.140625" customWidth="1"/>
+    <col min="10" max="10" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -2970,7 +2977,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>74</v>
       </c>
@@ -2996,7 +3003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>108</v>
       </c>
@@ -3045,117 +3052,117 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DC79B9-9C58-497E-9FD8-D3F2239E9BDC}">
   <dimension ref="A1:A22"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>101</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>109</v>
       </c>

</xml_diff>

<commit_message>
adjustments of the raw ammonia input
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\ammonia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{63D1B9E0-7B43-446D-9025-82534FC356E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2622E603-64E9-4248-8F95-220805F05EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="130">
   <si>
     <t>Unit</t>
   </si>
@@ -446,6 +446,24 @@
   </si>
   <si>
     <t>D</t>
+  </si>
+  <si>
+    <t>air_import</t>
+  </si>
+  <si>
+    <t>air_source</t>
+  </si>
+  <si>
+    <t>air</t>
+  </si>
+  <si>
+    <t>compression_raw_nh3</t>
+  </si>
+  <si>
+    <t>Compressor</t>
+  </si>
+  <si>
+    <t>raw_nh3</t>
   </si>
 </sst>
 </file>
@@ -476,7 +494,6 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -1442,8 +1459,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E5F8A7EB-52A6-4AC4-94D0-FF5952E382A3}" name="Table4" displayName="Table4" ref="A1:A22" totalsRowShown="0">
-  <autoFilter ref="A1:A22" xr:uid="{E5F8A7EB-52A6-4AC4-94D0-FF5952E382A3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E5F8A7EB-52A6-4AC4-94D0-FF5952E382A3}" name="Table4" displayName="Table4" ref="A1:A23" totalsRowShown="0">
+  <autoFilter ref="A1:A23" xr:uid="{E5F8A7EB-52A6-4AC4-94D0-FF5952E382A3}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{99EC3AFF-E76A-4BF2-94D0-13EEEC46286A}" name="object_type"/>
   </tableColumns>
@@ -1953,10 +1970,26 @@
       <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A9" s="10"/>
+      <c r="A9" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
-      <c r="A10" s="9"/>
+      <c r="A10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" s="10"/>
@@ -1986,7 +2019,7 @@
           <x14:formula1>
             <xm:f>Drop_Down!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>C12:C1048576 A11 B1:B8</xm:sqref>
+          <xm:sqref>C12:C1048576 A11 B1:B10</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -2160,7 +2193,9 @@
       <c r="H5" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="I5" s="4"/>
+      <c r="I5" s="4" t="s">
+        <v>110</v>
+      </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4">
         <v>5.8500000000000002E-3</v>
@@ -2171,7 +2206,9 @@
       <c r="O5" s="4">
         <v>1.76</v>
       </c>
-      <c r="P5" s="4"/>
+      <c r="P5" s="4">
+        <v>4.1662499999999998</v>
+      </c>
       <c r="Q5" s="4"/>
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
@@ -2184,26 +2221,26 @@
       <c r="C6" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="D6" s="3"/>
+      <c r="D6" t="s">
+        <v>126</v>
+      </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="H6" s="3" t="s">
-        <v>110</v>
-      </c>
+      <c r="H6" s="3"/>
       <c r="I6" s="3"/>
       <c r="J6" s="3"/>
-      <c r="K6" s="3"/>
+      <c r="K6">
+        <v>0.35</v>
+      </c>
       <c r="L6" s="3"/>
       <c r="M6" s="3"/>
-      <c r="N6" s="3">
-        <v>0.25</v>
-      </c>
-      <c r="O6" s="3">
-        <v>3.4482758620689657</v>
-      </c>
+      <c r="N6">
+        <v>2.7777777777777779E-3</v>
+      </c>
+      <c r="O6" s="3"/>
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
     </row>
@@ -2215,14 +2252,12 @@
         <v>101</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>73</v>
+        <v>129</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="E7" s="4" t="s">
-        <v>103</v>
-      </c>
+      <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
         <v>104</v>
@@ -2233,21 +2268,19 @@
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
       <c r="K7">
-        <v>17.867924528301888</v>
+        <v>52.631578947368425</v>
       </c>
       <c r="L7" s="4">
         <v>53.933348030570251</v>
       </c>
       <c r="M7" s="4"/>
       <c r="N7">
-        <v>1.1506682867557716</v>
+        <v>1</v>
       </c>
       <c r="O7" s="11">
-        <v>7.6203703703703694</v>
-      </c>
-      <c r="P7" s="4">
-        <v>21.657894736842106</v>
-      </c>
+        <v>6.8493150684931514</v>
+      </c>
+      <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
@@ -2279,21 +2312,56 @@
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
     </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C9" t="s">
+        <v>125</v>
+      </c>
+      <c r="G9" t="s">
+        <v>126</v>
+      </c>
+      <c r="N9">
+        <v>1</v>
+      </c>
+    </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A10" s="6"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="A10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B10" t="s">
+        <v>128</v>
+      </c>
+      <c r="C10" t="s">
+        <v>73</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>67</v>
+      </c>
       <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
+      <c r="G10" s="6" t="s">
+        <v>129</v>
+      </c>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
-      <c r="K10" s="6"/>
-      <c r="L10" s="6"/>
+      <c r="K10" s="6">
+        <v>1.3898000000000001E-2</v>
+      </c>
+      <c r="L10" s="6">
+        <v>18.181818181818183</v>
+      </c>
       <c r="M10" s="6"/>
-      <c r="N10" s="6"/>
+      <c r="N10" s="6">
+        <v>0.97360000000000002</v>
+      </c>
       <c r="O10" s="6"/>
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
@@ -2311,7 +2379,7 @@
           <x14:formula1>
             <xm:f>Drop_Down!$A:$A</xm:f>
           </x14:formula1>
-          <xm:sqref>B10 B1:B8</xm:sqref>
+          <xm:sqref>B1:B10</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3051,7 +3119,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DC79B9-9C58-497E-9FD8-D3F2239E9BDC}">
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
@@ -3167,6 +3235,11 @@
         <v>109</v>
       </c>
     </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>128</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
check approach and address issues
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\ammonia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2622E603-64E9-4248-8F95-220805F05EC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5495F943-49C0-452A-A06D-80474DD8BD59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
     <definedName name="IQ_YTD">3000</definedName>
     <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
   </definedNames>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="191028" concurrentManualCount="6"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="243" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="130">
   <si>
     <t>Unit</t>
   </si>
@@ -610,6 +610,12 @@
       </fill>
     </dxf>
     <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -626,14 +632,10 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79998168889431442"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
       <border diagonalUp="0" diagonalDown="0">
-        <left/>
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1222,6 +1224,42 @@
       </border>
     </dxf>
     <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1296,44 +1334,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1351,7 +1351,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}" name="Table1" displayName="Table1" ref="A1:R11" totalsRowShown="0">
   <autoFilter ref="A1:R11" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{88DF4E3A-CD2C-432F-B85D-4C82436680EB}" name="Unit" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{88DF4E3A-CD2C-432F-B85D-4C82436680EB}" name="Unit" dataDxfId="5"/>
     <tableColumn id="40" xr3:uid="{C2CFC5A4-5329-4F74-926A-18CEB18C062C}" name="Object_type"/>
     <tableColumn id="19" xr3:uid="{976E2DCC-BEF9-4E7C-96F4-92D75CC694A2}" name="unit_capacity"/>
     <tableColumn id="35" xr3:uid="{C3887B4E-C4A5-42AB-A92F-97AD44212E95}" name="mean_efficiency"/>
@@ -1366,8 +1366,8 @@
     <tableColumn id="12" xr3:uid="{F1A83AF0-CF23-4B00-9076-4E28DF8DAFD3}" name="fom_cost"/>
     <tableColumn id="21" xr3:uid="{400CD12D-8ADA-4557-B7CA-1464809EAFF0}" name="vom_cost"/>
     <tableColumn id="15" xr3:uid="{3F5A9F9C-E4A0-47A3-8DED-03601A5E69E7}" name="minimum_op_point"/>
-    <tableColumn id="38" xr3:uid="{957AF85B-8792-4643-A381-29FACAA69887}" name="resolution_output" dataDxfId="26"/>
-    <tableColumn id="39" xr3:uid="{BCE2350E-150B-4A7E-94BF-BB3BC7E31016}" name="demand" dataDxfId="25"/>
+    <tableColumn id="38" xr3:uid="{957AF85B-8792-4643-A381-29FACAA69887}" name="resolution_output" dataDxfId="4"/>
+    <tableColumn id="39" xr3:uid="{BCE2350E-150B-4A7E-94BF-BB3BC7E31016}" name="demand" dataDxfId="3"/>
     <tableColumn id="16" xr3:uid="{5F06ED78-6F41-4BEA-9209-36407E8BCFDC}" name="initial_units_on"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1375,26 +1375,26 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}" name="Table5" displayName="Table5" ref="A1:Q10" totalsRowShown="0" headerRowDxfId="24" dataDxfId="22" headerRowBorderDxfId="23" tableBorderDxfId="21" totalsRowBorderDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}" name="Table5" displayName="Table5" ref="A1:Q10" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
   <autoFilter ref="A1:Q10" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{2BE3E317-773B-4E82-9035-69A43C6CB21B}" name="Unit" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{22613EE0-390D-4B04-9A9B-6D5554D1C8ED}" name="Object_type" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{54CD83B6-B63A-4ABD-99BD-9ED391BFB078}" name="Input1" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{F183F72C-A42E-4046-9CA2-B23C4DD3765C}" name="Input2" dataDxfId="16"/>
-    <tableColumn id="7" xr3:uid="{CA468CF3-FA3A-4DED-8C1A-ED8385FD2167}" name="Input3" dataDxfId="15"/>
-    <tableColumn id="8" xr3:uid="{6C9174ED-453E-45B1-B2C9-DC69B7CB535A}" name="Input4" dataDxfId="14"/>
-    <tableColumn id="5" xr3:uid="{513A63E4-7BE3-4AF5-AC5E-11EB4AF0D7AD}" name="Output1" dataDxfId="13"/>
-    <tableColumn id="6" xr3:uid="{4623E738-60A2-497B-BD61-91A608129A61}" name="Output2" dataDxfId="12"/>
-    <tableColumn id="9" xr3:uid="{5596B30B-5CDD-4E38-8C15-9C5F774E9B1F}" name="Output3" dataDxfId="11"/>
-    <tableColumn id="10" xr3:uid="{CD6FCAF1-2543-4CF8-99F5-E24DBA2DEDC0}" name="Output4" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{88F2DAC4-E2C3-4C34-B709-2523E8BE5B1F}" name="Relation_In1_In2" dataDxfId="9"/>
-    <tableColumn id="14" xr3:uid="{3C190E97-FD9A-4F36-8EBF-717B1ECA00B1}" name="Relation_In1_In3" dataDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{043147D8-AE82-457E-8F19-EB4AE9D43B9E}" name="Relation_In1_In4" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{A190E492-7FDF-403D-B8AF-17448A48E47F}" name="Relation_In1_Out1" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{26E8D274-C985-4E20-8920-2BAC0A372552}" name="Relation_Out1_Out2" dataDxfId="5"/>
-    <tableColumn id="16" xr3:uid="{4E0BCAE8-11F8-4D98-AECC-86C8A3C2B5C1}" name="Relation_Out1_Out3" dataDxfId="4"/>
-    <tableColumn id="17" xr3:uid="{3C0369D5-4DD0-4B4B-9480-0C4665C0BC59}" name="Relation_Out1_Out4" dataDxfId="3"/>
+    <tableColumn id="1" xr3:uid="{2BE3E317-773B-4E82-9035-69A43C6CB21B}" name="Unit" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{22613EE0-390D-4B04-9A9B-6D5554D1C8ED}" name="Object_type" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{54CD83B6-B63A-4ABD-99BD-9ED391BFB078}" name="Input1" dataDxfId="20"/>
+    <tableColumn id="4" xr3:uid="{F183F72C-A42E-4046-9CA2-B23C4DD3765C}" name="Input2" dataDxfId="19"/>
+    <tableColumn id="7" xr3:uid="{CA468CF3-FA3A-4DED-8C1A-ED8385FD2167}" name="Input3" dataDxfId="18"/>
+    <tableColumn id="8" xr3:uid="{6C9174ED-453E-45B1-B2C9-DC69B7CB535A}" name="Input4" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{513A63E4-7BE3-4AF5-AC5E-11EB4AF0D7AD}" name="Output1" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{4623E738-60A2-497B-BD61-91A608129A61}" name="Output2" dataDxfId="15"/>
+    <tableColumn id="9" xr3:uid="{5596B30B-5CDD-4E38-8C15-9C5F774E9B1F}" name="Output3" dataDxfId="14"/>
+    <tableColumn id="10" xr3:uid="{CD6FCAF1-2543-4CF8-99F5-E24DBA2DEDC0}" name="Output4" dataDxfId="13"/>
+    <tableColumn id="11" xr3:uid="{88F2DAC4-E2C3-4C34-B709-2523E8BE5B1F}" name="Relation_In1_In2" dataDxfId="12"/>
+    <tableColumn id="14" xr3:uid="{3C190E97-FD9A-4F36-8EBF-717B1ECA00B1}" name="Relation_In1_In3" dataDxfId="11"/>
+    <tableColumn id="15" xr3:uid="{043147D8-AE82-457E-8F19-EB4AE9D43B9E}" name="Relation_In1_In4" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{A190E492-7FDF-403D-B8AF-17448A48E47F}" name="Relation_In1_Out1" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{26E8D274-C985-4E20-8920-2BAC0A372552}" name="Relation_Out1_Out2" dataDxfId="8"/>
+    <tableColumn id="16" xr3:uid="{4E0BCAE8-11F8-4D98-AECC-86C8A3C2B5C1}" name="Relation_Out1_Out3" dataDxfId="7"/>
+    <tableColumn id="17" xr3:uid="{3C0369D5-4DD0-4B4B-9480-0C4665C0BC59}" name="Relation_Out1_Out4" dataDxfId="6"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2270,9 +2270,7 @@
       <c r="K7">
         <v>52.631578947368425</v>
       </c>
-      <c r="L7" s="4">
-        <v>53.933348030570251</v>
-      </c>
+      <c r="L7" s="4"/>
       <c r="M7" s="4"/>
       <c r="N7">
         <v>1</v>
@@ -2637,6 +2635,36 @@
       <c r="G4" t="s">
         <v>32</v>
       </c>
+      <c r="H4">
+        <v>1000</v>
+      </c>
+      <c r="J4">
+        <v>1000</v>
+      </c>
+      <c r="K4">
+        <v>1000</v>
+      </c>
+      <c r="L4">
+        <v>1000</v>
+      </c>
+      <c r="M4">
+        <v>1000</v>
+      </c>
+      <c r="N4">
+        <v>1000</v>
+      </c>
+      <c r="R4">
+        <v>0.99983999999999995</v>
+      </c>
+      <c r="T4">
+        <v>0.99983999999999995</v>
+      </c>
+      <c r="U4">
+        <v>1.0958904109589041E-2</v>
+      </c>
+      <c r="Z4" t="s">
+        <v>54</v>
+      </c>
       <c r="AA4">
         <v>1</v>
       </c>
@@ -3084,6 +3112,12 @@
       <c r="D3" t="b">
         <v>1</v>
       </c>
+      <c r="E3">
+        <v>2640</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
       <c r="G3" t="s">
         <v>39</v>
       </c>

</xml_diff>

<commit_message>
remove dh connection from raw_product file
this will be implemented within the district heating function.
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\ammonia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5495F943-49C0-452A-A06D-80474DD8BD59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B467E2C4-1F71-4D4E-A330-F0E06CE8B525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="127">
   <si>
     <t>Unit</t>
   </si>
@@ -286,12 +286,6 @@
     <t>power_wholesale</t>
   </si>
   <si>
-    <t>pl_dh</t>
-  </si>
-  <si>
-    <t>dh</t>
-  </si>
-  <si>
     <t>water</t>
   </si>
   <si>
@@ -440,9 +434,6 @@
   </si>
   <si>
     <t>excess_heat</t>
-  </si>
-  <si>
-    <t>heat</t>
   </si>
   <si>
     <t>D</t>
@@ -599,21 +590,12 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="none">
           <fgColor indexed="64"/>
           <bgColor auto="1"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -632,10 +614,14 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
       <border diagonalUp="0" diagonalDown="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
+        <left/>
         <right/>
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1224,42 +1210,6 @@
       </border>
     </dxf>
     <dxf>
-      <font>
-        <b val="0"/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79998168889431442"/>
-          <bgColor theme="4" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-      <border diagonalUp="0" diagonalDown="0">
-        <left/>
-        <right/>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-        <vertical/>
-        <horizontal/>
-      </border>
-    </dxf>
-    <dxf>
       <border outline="0">
         <top style="thin">
           <color theme="4" tint="0.39997558519241921"/>
@@ -1334,6 +1284,47 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1351,7 +1342,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}" name="Table1" displayName="Table1" ref="A1:R11" totalsRowShown="0">
   <autoFilter ref="A1:R11" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{88DF4E3A-CD2C-432F-B85D-4C82436680EB}" name="Unit" dataDxfId="5"/>
+    <tableColumn id="1" xr3:uid="{88DF4E3A-CD2C-432F-B85D-4C82436680EB}" name="Unit" dataDxfId="26"/>
     <tableColumn id="40" xr3:uid="{C2CFC5A4-5329-4F74-926A-18CEB18C062C}" name="Object_type"/>
     <tableColumn id="19" xr3:uid="{976E2DCC-BEF9-4E7C-96F4-92D75CC694A2}" name="unit_capacity"/>
     <tableColumn id="35" xr3:uid="{C3887B4E-C4A5-42AB-A92F-97AD44212E95}" name="mean_efficiency"/>
@@ -1366,8 +1357,8 @@
     <tableColumn id="12" xr3:uid="{F1A83AF0-CF23-4B00-9076-4E28DF8DAFD3}" name="fom_cost"/>
     <tableColumn id="21" xr3:uid="{400CD12D-8ADA-4557-B7CA-1464809EAFF0}" name="vom_cost"/>
     <tableColumn id="15" xr3:uid="{3F5A9F9C-E4A0-47A3-8DED-03601A5E69E7}" name="minimum_op_point"/>
-    <tableColumn id="38" xr3:uid="{957AF85B-8792-4643-A381-29FACAA69887}" name="resolution_output" dataDxfId="4"/>
-    <tableColumn id="39" xr3:uid="{BCE2350E-150B-4A7E-94BF-BB3BC7E31016}" name="demand" dataDxfId="3"/>
+    <tableColumn id="38" xr3:uid="{957AF85B-8792-4643-A381-29FACAA69887}" name="resolution_output" dataDxfId="25"/>
+    <tableColumn id="39" xr3:uid="{BCE2350E-150B-4A7E-94BF-BB3BC7E31016}" name="demand" dataDxfId="24"/>
     <tableColumn id="16" xr3:uid="{5F06ED78-6F41-4BEA-9209-36407E8BCFDC}" name="initial_units_on"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1375,34 +1366,34 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}" name="Table5" displayName="Table5" ref="A1:Q10" totalsRowShown="0" headerRowDxfId="27" dataDxfId="25" headerRowBorderDxfId="26" tableBorderDxfId="24" totalsRowBorderDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}" name="Table5" displayName="Table5" ref="A1:Q10" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="19">
   <autoFilter ref="A1:Q10" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{2BE3E317-773B-4E82-9035-69A43C6CB21B}" name="Unit" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{22613EE0-390D-4B04-9A9B-6D5554D1C8ED}" name="Object_type" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{54CD83B6-B63A-4ABD-99BD-9ED391BFB078}" name="Input1" dataDxfId="20"/>
-    <tableColumn id="4" xr3:uid="{F183F72C-A42E-4046-9CA2-B23C4DD3765C}" name="Input2" dataDxfId="19"/>
-    <tableColumn id="7" xr3:uid="{CA468CF3-FA3A-4DED-8C1A-ED8385FD2167}" name="Input3" dataDxfId="18"/>
-    <tableColumn id="8" xr3:uid="{6C9174ED-453E-45B1-B2C9-DC69B7CB535A}" name="Input4" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{513A63E4-7BE3-4AF5-AC5E-11EB4AF0D7AD}" name="Output1" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{4623E738-60A2-497B-BD61-91A608129A61}" name="Output2" dataDxfId="15"/>
-    <tableColumn id="9" xr3:uid="{5596B30B-5CDD-4E38-8C15-9C5F774E9B1F}" name="Output3" dataDxfId="14"/>
-    <tableColumn id="10" xr3:uid="{CD6FCAF1-2543-4CF8-99F5-E24DBA2DEDC0}" name="Output4" dataDxfId="13"/>
-    <tableColumn id="11" xr3:uid="{88F2DAC4-E2C3-4C34-B709-2523E8BE5B1F}" name="Relation_In1_In2" dataDxfId="12"/>
-    <tableColumn id="14" xr3:uid="{3C190E97-FD9A-4F36-8EBF-717B1ECA00B1}" name="Relation_In1_In3" dataDxfId="11"/>
-    <tableColumn id="15" xr3:uid="{043147D8-AE82-457E-8F19-EB4AE9D43B9E}" name="Relation_In1_In4" dataDxfId="10"/>
-    <tableColumn id="12" xr3:uid="{A190E492-7FDF-403D-B8AF-17448A48E47F}" name="Relation_In1_Out1" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{26E8D274-C985-4E20-8920-2BAC0A372552}" name="Relation_Out1_Out2" dataDxfId="8"/>
-    <tableColumn id="16" xr3:uid="{4E0BCAE8-11F8-4D98-AECC-86C8A3C2B5C1}" name="Relation_Out1_Out3" dataDxfId="7"/>
-    <tableColumn id="17" xr3:uid="{3C0369D5-4DD0-4B4B-9480-0C4665C0BC59}" name="Relation_Out1_Out4" dataDxfId="6"/>
+    <tableColumn id="1" xr3:uid="{2BE3E317-773B-4E82-9035-69A43C6CB21B}" name="Unit" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{22613EE0-390D-4B04-9A9B-6D5554D1C8ED}" name="Object_type" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{54CD83B6-B63A-4ABD-99BD-9ED391BFB078}" name="Input1" dataDxfId="16"/>
+    <tableColumn id="4" xr3:uid="{F183F72C-A42E-4046-9CA2-B23C4DD3765C}" name="Input2" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{CA468CF3-FA3A-4DED-8C1A-ED8385FD2167}" name="Input3" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{6C9174ED-453E-45B1-B2C9-DC69B7CB535A}" name="Input4" dataDxfId="13"/>
+    <tableColumn id="5" xr3:uid="{513A63E4-7BE3-4AF5-AC5E-11EB4AF0D7AD}" name="Output1" dataDxfId="12"/>
+    <tableColumn id="6" xr3:uid="{4623E738-60A2-497B-BD61-91A608129A61}" name="Output2" dataDxfId="11"/>
+    <tableColumn id="9" xr3:uid="{5596B30B-5CDD-4E38-8C15-9C5F774E9B1F}" name="Output3" dataDxfId="10"/>
+    <tableColumn id="10" xr3:uid="{CD6FCAF1-2543-4CF8-99F5-E24DBA2DEDC0}" name="Output4" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{88F2DAC4-E2C3-4C34-B709-2523E8BE5B1F}" name="Relation_In1_In2" dataDxfId="8"/>
+    <tableColumn id="14" xr3:uid="{3C190E97-FD9A-4F36-8EBF-717B1ECA00B1}" name="Relation_In1_In3" dataDxfId="7"/>
+    <tableColumn id="15" xr3:uid="{043147D8-AE82-457E-8F19-EB4AE9D43B9E}" name="Relation_In1_In4" dataDxfId="6"/>
+    <tableColumn id="12" xr3:uid="{A190E492-7FDF-403D-B8AF-17448A48E47F}" name="Relation_In1_Out1" dataDxfId="5"/>
+    <tableColumn id="13" xr3:uid="{26E8D274-C985-4E20-8920-2BAC0A372552}" name="Relation_Out1_Out2" dataDxfId="4"/>
+    <tableColumn id="16" xr3:uid="{4E0BCAE8-11F8-4D98-AECC-86C8A3C2B5C1}" name="Relation_Out1_Out3" dataDxfId="3"/>
+    <tableColumn id="17" xr3:uid="{3C0369D5-4DD0-4B4B-9480-0C4665C0BC59}" name="Relation_Out1_Out4" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{856854C3-DC05-4AB8-91B8-0E52D9C11DBC}" name="Table13" displayName="Table13" ref="A1:AA11" totalsRowShown="0">
-  <autoFilter ref="A1:AA11" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{856854C3-DC05-4AB8-91B8-0E52D9C11DBC}" name="Table13" displayName="Table13" ref="A1:AA10" totalsRowShown="0">
+  <autoFilter ref="A1:AA10" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
   <tableColumns count="27">
     <tableColumn id="1" xr3:uid="{26B0CA71-1EA9-44CF-8E6D-31054ECA99A6}" name="Connection"/>
     <tableColumn id="26" xr3:uid="{E67F4435-EF76-417C-B715-53719E5FB41F}" name="Object_type"/>
@@ -1410,7 +1401,7 @@
     <tableColumn id="3" xr3:uid="{0B221EED-10BC-4C34-AC5E-37A826B1E8AE}" name="Input2"/>
     <tableColumn id="4" xr3:uid="{13095F0A-BCF6-40A3-B029-60B11214B154}" name="Output1"/>
     <tableColumn id="5" xr3:uid="{4C6B3E52-C4A2-4D67-B50B-9DAA089E0399}" name="Output2"/>
-    <tableColumn id="22" xr3:uid="{551A8663-4680-4147-9E64-4B9A8EA76642}" name="Connection_type" dataDxfId="2"/>
+    <tableColumn id="22" xr3:uid="{551A8663-4680-4147-9E64-4B9A8EA76642}" name="Connection_type" dataDxfId="1"/>
     <tableColumn id="6" xr3:uid="{5DF4D35D-AD4C-4648-BC90-B2BA8F975A09}" name="Cap_Input1_existing"/>
     <tableColumn id="15" xr3:uid="{C0BCA9EF-0E20-40E5-9820-0EA6AB1DE457}" name="Cap_Input1_max"/>
     <tableColumn id="14" xr3:uid="{D4F16D16-99DE-47DA-B08A-6DD56FEBC7A4}" name="Cap_Input2_existing"/>
@@ -1429,7 +1420,7 @@
     <tableColumn id="21" xr3:uid="{EC2CC790-C17D-4744-A981-3984808E5B33}" name="vom_cost_Input2"/>
     <tableColumn id="24" xr3:uid="{41B338E4-2058-41E9-8000-97D77450FBC3}" name="vom_cost_Output1"/>
     <tableColumn id="25" xr3:uid="{DDAFCF0A-1EF1-4B7B-9742-01F9FA7A22E5}" name="vom_cost_Output2"/>
-    <tableColumn id="29" xr3:uid="{79DE3A19-CED6-47DE-AEF5-F6BB2D320F24}" name="connection_investment_tech_lifetime" dataDxfId="1"/>
+    <tableColumn id="29" xr3:uid="{79DE3A19-CED6-47DE-AEF5-F6BB2D320F24}" name="connection_investment_tech_lifetime" dataDxfId="0"/>
     <tableColumn id="30" xr3:uid="{09434E4A-7BF5-4547-9708-EA3F0F7ADC8E}" name="initial_connections_invested_available"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1440,8 +1431,8 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{070C7B69-9214-47B9-93F0-C6C6118ED7CC}" name="Table134" displayName="Table134" ref="A1:K5" totalsRowShown="0">
   <autoFilter ref="A1:K5" xr:uid="{070C7B69-9214-47B9-93F0-C6C6118ED7CC}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{59CF1CEF-E7FA-4B7F-9443-D4A6EAAB7A8F}" name="Storage" dataDxfId="0">
-      <calculatedColumnFormula array="1">_xlfn._xlws.FILTER(Connections!A2:A100,ISNUMBER(FIND("storage",Connections!A2:A100)))</calculatedColumnFormula>
+    <tableColumn id="1" xr3:uid="{59CF1CEF-E7FA-4B7F-9443-D4A6EAAB7A8F}" name="Storage" dataDxfId="27">
+      <calculatedColumnFormula array="1">_xlfn._xlws.FILTER(Connections!A2:A99,ISNUMBER(FIND("storage",Connections!A2:A99)))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{8C29206C-8DC6-44DB-A8D1-3D5625C277AD}" name="Object_type"/>
     <tableColumn id="4" xr3:uid="{AEAA1B51-84C1-491F-81D5-7757B30BDCCD}" name="value_before"/>
@@ -1796,7 +1787,7 @@
         <v>42</v>
       </c>
       <c r="C1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D1" t="s">
         <v>12</v>
@@ -1805,16 +1796,16 @@
         <v>13</v>
       </c>
       <c r="F1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="G1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="H1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="I1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="J1" t="s">
         <v>61</v>
@@ -1841,7 +1832,7 @@
         <v>41</v>
       </c>
       <c r="R1" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
@@ -1852,40 +1843,40 @@
         <v>43</v>
       </c>
       <c r="C2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A3" s="10" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B3" t="s">
         <v>59</v>
       </c>
       <c r="C3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" s="9" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
         <v>60</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A5" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B5" t="s">
         <v>57</v>
@@ -1907,13 +1898,13 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" s="9" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="O6">
         <v>0.4</v>
@@ -1923,16 +1914,16 @@
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
+        <v>100</v>
+      </c>
+      <c r="B7" t="s">
+        <v>99</v>
+      </c>
+      <c r="C7" t="s">
         <v>102</v>
       </c>
-      <c r="B7" t="s">
-        <v>101</v>
-      </c>
-      <c r="C7" t="s">
-        <v>104</v>
-      </c>
       <c r="E7" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F7">
         <v>0.5</v>
@@ -1950,7 +1941,7 @@
         <v>0.2</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="Q7" s="2">
         <v>20</v>
@@ -1958,37 +1949,37 @@
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" s="9" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B8" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
@@ -2058,10 +2049,10 @@
         <v>2</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G1" s="5" t="s">
         <v>3</v>
@@ -2070,31 +2061,31 @@
         <v>4</v>
       </c>
       <c r="I1" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="J1" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="K1" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="J1" s="5" t="s">
+      <c r="L1" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="K1" s="5" t="s">
+      <c r="M1" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>84</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="P1" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="O1" s="5" t="s">
+      <c r="Q1" s="5" t="s">
         <v>87</v>
-      </c>
-      <c r="P1" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="Q1" s="5" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
@@ -2109,7 +2100,7 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="H2" s="3"/>
       <c r="I2" s="7"/>
@@ -2124,7 +2115,7 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B3" s="4" t="s">
         <v>59</v>
@@ -2134,7 +2125,7 @@
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
       <c r="G3" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="H3" s="4"/>
       <c r="I3" s="4"/>
@@ -2149,7 +2140,7 @@
     </row>
     <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B4" t="s">
         <v>60</v>
@@ -2159,7 +2150,7 @@
       <c r="E4" s="3"/>
       <c r="F4" s="3"/>
       <c r="G4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H4" s="3"/>
       <c r="I4" s="3"/>
@@ -2174,7 +2165,7 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B5" s="4" t="s">
         <v>57</v>
@@ -2183,18 +2174,18 @@
         <v>67</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E5" s="4"/>
       <c r="F5" s="4"/>
       <c r="G5" s="4" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="H5" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I5" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J5" s="4"/>
       <c r="K5" s="4">
@@ -2213,21 +2204,21 @@
     </row>
     <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C6" s="3" t="s">
         <v>67</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="E6" s="3"/>
       <c r="F6" s="3"/>
       <c r="G6" s="3" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H6" s="3"/>
       <c r="I6" s="3"/>
@@ -2246,13 +2237,13 @@
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="D7" s="4" t="s">
         <v>67</v>
@@ -2260,10 +2251,10 @@
       <c r="E7" s="4"/>
       <c r="F7" s="4"/>
       <c r="G7" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="I7" s="4"/>
       <c r="J7" s="4"/>
@@ -2283,19 +2274,19 @@
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="4"/>
       <c r="F8" s="4"/>
       <c r="G8" s="4" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
@@ -2312,16 +2303,16 @@
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="10" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B9" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="G9" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="N9">
         <v>1</v>
@@ -2329,23 +2320,23 @@
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B10" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D10" s="6" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>67</v>
       </c>
       <c r="F10" s="6"/>
       <c r="G10" s="6" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
@@ -2387,7 +2378,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C870BDA0-9E4C-481D-87BE-9D47789809C8}">
-  <dimension ref="A1:AA11"/>
+  <dimension ref="A1:AA10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
@@ -2559,22 +2550,22 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B3" t="s">
         <v>50</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="F3" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="G3" t="s">
         <v>32</v>
@@ -2615,22 +2606,22 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="E4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G4" t="s">
         <v>32</v>
@@ -2671,16 +2662,22 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>70</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C5" t="s">
-        <v>122</v>
+        <v>69</v>
+      </c>
+      <c r="D5" t="s">
+        <v>110</v>
       </c>
       <c r="E5" t="s">
-        <v>71</v>
+        <v>110</v>
+      </c>
+      <c r="F5" t="s">
+        <v>69</v>
       </c>
       <c r="G5" t="s">
         <v>32</v>
@@ -2691,11 +2688,26 @@
       <c r="I5">
         <v>1000</v>
       </c>
+      <c r="J5">
+        <v>1000</v>
+      </c>
+      <c r="K5">
+        <v>1000</v>
+      </c>
       <c r="L5">
         <v>1000</v>
       </c>
       <c r="M5">
         <v>1000</v>
+      </c>
+      <c r="N5">
+        <v>1000</v>
+      </c>
+      <c r="O5">
+        <v>1000</v>
+      </c>
+      <c r="R5">
+        <v>1</v>
       </c>
       <c r="T5">
         <v>1</v>
@@ -2709,22 +2721,16 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
         <v>51</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D6" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="E6" t="s">
-        <v>112</v>
-      </c>
-      <c r="F6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G6" t="s">
         <v>32</v>
@@ -2735,26 +2741,11 @@
       <c r="I6">
         <v>1000</v>
       </c>
-      <c r="J6">
-        <v>1000</v>
-      </c>
-      <c r="K6">
-        <v>1000</v>
-      </c>
       <c r="L6">
         <v>1000</v>
       </c>
       <c r="M6">
         <v>1000</v>
-      </c>
-      <c r="N6">
-        <v>1000</v>
-      </c>
-      <c r="O6">
-        <v>1000</v>
-      </c>
-      <c r="R6">
-        <v>1</v>
       </c>
       <c r="T6">
         <v>1</v>
@@ -2768,16 +2759,22 @@
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
         <v>51</v>
       </c>
       <c r="C7" t="s">
-        <v>112</v>
+        <v>69</v>
+      </c>
+      <c r="D7" t="s">
+        <v>111</v>
       </c>
       <c r="E7" t="s">
-        <v>67</v>
+        <v>111</v>
+      </c>
+      <c r="F7" t="s">
+        <v>69</v>
       </c>
       <c r="G7" t="s">
         <v>32</v>
@@ -2788,11 +2785,26 @@
       <c r="I7">
         <v>1000</v>
       </c>
+      <c r="J7">
+        <v>1000</v>
+      </c>
+      <c r="K7">
+        <v>1000</v>
+      </c>
       <c r="L7">
         <v>1000</v>
       </c>
       <c r="M7">
         <v>1000</v>
+      </c>
+      <c r="N7">
+        <v>1000</v>
+      </c>
+      <c r="O7">
+        <v>1000</v>
+      </c>
+      <c r="R7">
+        <v>1</v>
       </c>
       <c r="T7">
         <v>1</v>
@@ -2806,22 +2818,16 @@
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B8" t="s">
         <v>51</v>
       </c>
       <c r="C8" t="s">
-        <v>69</v>
-      </c>
-      <c r="D8" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="E8" t="s">
-        <v>113</v>
-      </c>
-      <c r="F8" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G8" t="s">
         <v>32</v>
@@ -2832,26 +2838,11 @@
       <c r="I8">
         <v>1000</v>
       </c>
-      <c r="J8">
-        <v>1000</v>
-      </c>
-      <c r="K8">
-        <v>1000</v>
-      </c>
       <c r="L8">
         <v>1000</v>
       </c>
       <c r="M8">
         <v>1000</v>
-      </c>
-      <c r="N8">
-        <v>1000</v>
-      </c>
-      <c r="O8">
-        <v>1000</v>
-      </c>
-      <c r="R8">
-        <v>1</v>
       </c>
       <c r="T8">
         <v>1</v>
@@ -2865,16 +2856,22 @@
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B9" t="s">
         <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>113</v>
+        <v>69</v>
+      </c>
+      <c r="D9" t="s">
+        <v>112</v>
       </c>
       <c r="E9" t="s">
-        <v>67</v>
+        <v>112</v>
+      </c>
+      <c r="F9" t="s">
+        <v>69</v>
       </c>
       <c r="G9" t="s">
         <v>32</v>
@@ -2885,11 +2882,26 @@
       <c r="I9">
         <v>1000</v>
       </c>
+      <c r="J9">
+        <v>1000</v>
+      </c>
+      <c r="K9">
+        <v>1000</v>
+      </c>
       <c r="L9">
         <v>1000</v>
       </c>
       <c r="M9">
         <v>1000</v>
+      </c>
+      <c r="N9">
+        <v>1000</v>
+      </c>
+      <c r="O9">
+        <v>1000</v>
+      </c>
+      <c r="R9">
+        <v>1</v>
       </c>
       <c r="T9">
         <v>1</v>
@@ -2903,22 +2915,16 @@
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B10" t="s">
         <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>69</v>
-      </c>
-      <c r="D10" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E10" t="s">
-        <v>114</v>
-      </c>
-      <c r="F10" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="G10" t="s">
         <v>32</v>
@@ -2929,26 +2935,11 @@
       <c r="I10">
         <v>1000</v>
       </c>
-      <c r="J10">
-        <v>1000</v>
-      </c>
-      <c r="K10">
-        <v>1000</v>
-      </c>
       <c r="L10">
         <v>1000</v>
       </c>
       <c r="M10">
         <v>1000</v>
-      </c>
-      <c r="N10">
-        <v>1000</v>
-      </c>
-      <c r="O10">
-        <v>1000</v>
-      </c>
-      <c r="R10">
-        <v>1</v>
       </c>
       <c r="T10">
         <v>1</v>
@@ -2957,44 +2948,6 @@
         <v>55</v>
       </c>
       <c r="AA10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>120</v>
-      </c>
-      <c r="B11" t="s">
-        <v>51</v>
-      </c>
-      <c r="C11" t="s">
-        <v>114</v>
-      </c>
-      <c r="E11" t="s">
-        <v>67</v>
-      </c>
-      <c r="G11" t="s">
-        <v>32</v>
-      </c>
-      <c r="H11">
-        <v>1000</v>
-      </c>
-      <c r="I11">
-        <v>1000</v>
-      </c>
-      <c r="L11">
-        <v>1000</v>
-      </c>
-      <c r="M11">
-        <v>1000</v>
-      </c>
-      <c r="T11">
-        <v>1</v>
-      </c>
-      <c r="Z11" t="s">
-        <v>55</v>
-      </c>
-      <c r="AA11">
         <v>1</v>
       </c>
     </row>
@@ -3012,7 +2965,7 @@
           <x14:formula1>
             <xm:f>Drop_Down!$A$2:$A$60</xm:f>
           </x14:formula1>
-          <xm:sqref>B2:B100</xm:sqref>
+          <xm:sqref>B2:B99</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -3075,7 +3028,7 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B2" t="s">
         <v>47</v>
@@ -3101,10 +3054,10 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B3" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -3201,7 +3154,7 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.3">
@@ -3231,7 +3184,7 @@
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.3">
@@ -3251,27 +3204,27 @@
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
bug fix and update raw input data for methanol
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/ammonia/Model_Data_Base_ammonia.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B467E2C4-1F71-4D4E-A330-F0E06CE8B525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -53,7 +53,7 @@
     <definedName name="IQ_YTD">3000</definedName>
     <definedName name="IQ_YTDMONTH" hidden="1">130000</definedName>
   </definedNames>
-  <calcPr calcId="191028" concurrentManualCount="6"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -590,14 +590,6 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <fill>
-        <patternFill patternType="none">
-          <fgColor indexed="64"/>
-          <bgColor auto="1"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
       <font>
         <b val="0"/>
         <i val="0"/>
@@ -1325,6 +1317,14 @@
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1342,7 +1342,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}" name="Table1" displayName="Table1" ref="A1:R11" totalsRowShown="0">
   <autoFilter ref="A1:R11" xr:uid="{A55D93BB-3EF1-4249-80C0-A8E75E738393}"/>
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{88DF4E3A-CD2C-432F-B85D-4C82436680EB}" name="Unit" dataDxfId="26"/>
+    <tableColumn id="1" xr3:uid="{88DF4E3A-CD2C-432F-B85D-4C82436680EB}" name="Unit" dataDxfId="25"/>
     <tableColumn id="40" xr3:uid="{C2CFC5A4-5329-4F74-926A-18CEB18C062C}" name="Object_type"/>
     <tableColumn id="19" xr3:uid="{976E2DCC-BEF9-4E7C-96F4-92D75CC694A2}" name="unit_capacity"/>
     <tableColumn id="35" xr3:uid="{C3887B4E-C4A5-42AB-A92F-97AD44212E95}" name="mean_efficiency"/>
@@ -1357,8 +1357,8 @@
     <tableColumn id="12" xr3:uid="{F1A83AF0-CF23-4B00-9076-4E28DF8DAFD3}" name="fom_cost"/>
     <tableColumn id="21" xr3:uid="{400CD12D-8ADA-4557-B7CA-1464809EAFF0}" name="vom_cost"/>
     <tableColumn id="15" xr3:uid="{3F5A9F9C-E4A0-47A3-8DED-03601A5E69E7}" name="minimum_op_point"/>
-    <tableColumn id="38" xr3:uid="{957AF85B-8792-4643-A381-29FACAA69887}" name="resolution_output" dataDxfId="25"/>
-    <tableColumn id="39" xr3:uid="{BCE2350E-150B-4A7E-94BF-BB3BC7E31016}" name="demand" dataDxfId="24"/>
+    <tableColumn id="38" xr3:uid="{957AF85B-8792-4643-A381-29FACAA69887}" name="resolution_output" dataDxfId="24"/>
+    <tableColumn id="39" xr3:uid="{BCE2350E-150B-4A7E-94BF-BB3BC7E31016}" name="demand" dataDxfId="23"/>
     <tableColumn id="16" xr3:uid="{5F06ED78-6F41-4BEA-9209-36407E8BCFDC}" name="initial_units_on"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1366,26 +1366,26 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}" name="Table5" displayName="Table5" ref="A1:Q10" totalsRowShown="0" headerRowDxfId="23" dataDxfId="21" headerRowBorderDxfId="22" tableBorderDxfId="20" totalsRowBorderDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}" name="Table5" displayName="Table5" ref="A1:Q10" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19" totalsRowBorderDxfId="18">
   <autoFilter ref="A1:Q10" xr:uid="{C1664CC4-80CB-414D-BAFE-57FF9635D79F}"/>
   <tableColumns count="17">
-    <tableColumn id="1" xr3:uid="{2BE3E317-773B-4E82-9035-69A43C6CB21B}" name="Unit" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{22613EE0-390D-4B04-9A9B-6D5554D1C8ED}" name="Object_type" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{54CD83B6-B63A-4ABD-99BD-9ED391BFB078}" name="Input1" dataDxfId="16"/>
-    <tableColumn id="4" xr3:uid="{F183F72C-A42E-4046-9CA2-B23C4DD3765C}" name="Input2" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{CA468CF3-FA3A-4DED-8C1A-ED8385FD2167}" name="Input3" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{6C9174ED-453E-45B1-B2C9-DC69B7CB535A}" name="Input4" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{513A63E4-7BE3-4AF5-AC5E-11EB4AF0D7AD}" name="Output1" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{4623E738-60A2-497B-BD61-91A608129A61}" name="Output2" dataDxfId="11"/>
-    <tableColumn id="9" xr3:uid="{5596B30B-5CDD-4E38-8C15-9C5F774E9B1F}" name="Output3" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{CD6FCAF1-2543-4CF8-99F5-E24DBA2DEDC0}" name="Output4" dataDxfId="9"/>
-    <tableColumn id="11" xr3:uid="{88F2DAC4-E2C3-4C34-B709-2523E8BE5B1F}" name="Relation_In1_In2" dataDxfId="8"/>
-    <tableColumn id="14" xr3:uid="{3C190E97-FD9A-4F36-8EBF-717B1ECA00B1}" name="Relation_In1_In3" dataDxfId="7"/>
-    <tableColumn id="15" xr3:uid="{043147D8-AE82-457E-8F19-EB4AE9D43B9E}" name="Relation_In1_In4" dataDxfId="6"/>
-    <tableColumn id="12" xr3:uid="{A190E492-7FDF-403D-B8AF-17448A48E47F}" name="Relation_In1_Out1" dataDxfId="5"/>
-    <tableColumn id="13" xr3:uid="{26E8D274-C985-4E20-8920-2BAC0A372552}" name="Relation_Out1_Out2" dataDxfId="4"/>
-    <tableColumn id="16" xr3:uid="{4E0BCAE8-11F8-4D98-AECC-86C8A3C2B5C1}" name="Relation_Out1_Out3" dataDxfId="3"/>
-    <tableColumn id="17" xr3:uid="{3C0369D5-4DD0-4B4B-9480-0C4665C0BC59}" name="Relation_Out1_Out4" dataDxfId="2"/>
+    <tableColumn id="1" xr3:uid="{2BE3E317-773B-4E82-9035-69A43C6CB21B}" name="Unit" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{22613EE0-390D-4B04-9A9B-6D5554D1C8ED}" name="Object_type" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{54CD83B6-B63A-4ABD-99BD-9ED391BFB078}" name="Input1" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{F183F72C-A42E-4046-9CA2-B23C4DD3765C}" name="Input2" dataDxfId="14"/>
+    <tableColumn id="7" xr3:uid="{CA468CF3-FA3A-4DED-8C1A-ED8385FD2167}" name="Input3" dataDxfId="13"/>
+    <tableColumn id="8" xr3:uid="{6C9174ED-453E-45B1-B2C9-DC69B7CB535A}" name="Input4" dataDxfId="12"/>
+    <tableColumn id="5" xr3:uid="{513A63E4-7BE3-4AF5-AC5E-11EB4AF0D7AD}" name="Output1" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{4623E738-60A2-497B-BD61-91A608129A61}" name="Output2" dataDxfId="10"/>
+    <tableColumn id="9" xr3:uid="{5596B30B-5CDD-4E38-8C15-9C5F774E9B1F}" name="Output3" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{CD6FCAF1-2543-4CF8-99F5-E24DBA2DEDC0}" name="Output4" dataDxfId="8"/>
+    <tableColumn id="11" xr3:uid="{88F2DAC4-E2C3-4C34-B709-2523E8BE5B1F}" name="Relation_In1_In2" dataDxfId="7"/>
+    <tableColumn id="14" xr3:uid="{3C190E97-FD9A-4F36-8EBF-717B1ECA00B1}" name="Relation_In1_In3" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{043147D8-AE82-457E-8F19-EB4AE9D43B9E}" name="Relation_In1_In4" dataDxfId="5"/>
+    <tableColumn id="12" xr3:uid="{A190E492-7FDF-403D-B8AF-17448A48E47F}" name="Relation_In1_Out1" dataDxfId="4"/>
+    <tableColumn id="13" xr3:uid="{26E8D274-C985-4E20-8920-2BAC0A372552}" name="Relation_Out1_Out2" dataDxfId="3"/>
+    <tableColumn id="16" xr3:uid="{4E0BCAE8-11F8-4D98-AECC-86C8A3C2B5C1}" name="Relation_Out1_Out3" dataDxfId="2"/>
+    <tableColumn id="17" xr3:uid="{3C0369D5-4DD0-4B4B-9480-0C4665C0BC59}" name="Relation_Out1_Out4" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1401,7 +1401,7 @@
     <tableColumn id="3" xr3:uid="{0B221EED-10BC-4C34-AC5E-37A826B1E8AE}" name="Input2"/>
     <tableColumn id="4" xr3:uid="{13095F0A-BCF6-40A3-B029-60B11214B154}" name="Output1"/>
     <tableColumn id="5" xr3:uid="{4C6B3E52-C4A2-4D67-B50B-9DAA089E0399}" name="Output2"/>
-    <tableColumn id="22" xr3:uid="{551A8663-4680-4147-9E64-4B9A8EA76642}" name="Connection_type" dataDxfId="1"/>
+    <tableColumn id="22" xr3:uid="{551A8663-4680-4147-9E64-4B9A8EA76642}" name="Connection_type" dataDxfId="27"/>
     <tableColumn id="6" xr3:uid="{5DF4D35D-AD4C-4648-BC90-B2BA8F975A09}" name="Cap_Input1_existing"/>
     <tableColumn id="15" xr3:uid="{C0BCA9EF-0E20-40E5-9820-0EA6AB1DE457}" name="Cap_Input1_max"/>
     <tableColumn id="14" xr3:uid="{D4F16D16-99DE-47DA-B08A-6DD56FEBC7A4}" name="Cap_Input2_existing"/>
@@ -1420,7 +1420,7 @@
     <tableColumn id="21" xr3:uid="{EC2CC790-C17D-4744-A981-3984808E5B33}" name="vom_cost_Input2"/>
     <tableColumn id="24" xr3:uid="{41B338E4-2058-41E9-8000-97D77450FBC3}" name="vom_cost_Output1"/>
     <tableColumn id="25" xr3:uid="{DDAFCF0A-1EF1-4B7B-9742-01F9FA7A22E5}" name="vom_cost_Output2"/>
-    <tableColumn id="29" xr3:uid="{79DE3A19-CED6-47DE-AEF5-F6BB2D320F24}" name="connection_investment_tech_lifetime" dataDxfId="0"/>
+    <tableColumn id="29" xr3:uid="{79DE3A19-CED6-47DE-AEF5-F6BB2D320F24}" name="connection_investment_tech_lifetime" dataDxfId="26"/>
     <tableColumn id="30" xr3:uid="{09434E4A-7BF5-4547-9708-EA3F0F7ADC8E}" name="initial_connections_invested_available"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1431,7 +1431,7 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{070C7B69-9214-47B9-93F0-C6C6118ED7CC}" name="Table134" displayName="Table134" ref="A1:K5" totalsRowShown="0">
   <autoFilter ref="A1:K5" xr:uid="{070C7B69-9214-47B9-93F0-C6C6118ED7CC}"/>
   <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{59CF1CEF-E7FA-4B7F-9443-D4A6EAAB7A8F}" name="Storage" dataDxfId="27">
+    <tableColumn id="1" xr3:uid="{59CF1CEF-E7FA-4B7F-9443-D4A6EAAB7A8F}" name="Storage" dataDxfId="0">
       <calculatedColumnFormula array="1">_xlfn._xlws.FILTER(Connections!A2:A99,ISNUMBER(FIND("storage",Connections!A2:A99)))</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="8" xr3:uid="{8C29206C-8DC6-44DB-A8D1-3D5625C277AD}" name="Object_type"/>
@@ -1757,29 +1757,29 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576C757C-091A-46DF-949E-B17661031FDE}">
   <dimension ref="A1:R12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.6328125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.08984375" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="11.6640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="21.109375" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="19.6640625" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.08984375" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.6328125" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="11.453125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="11.6328125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="21.08984375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="19.6328125" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
@@ -1835,7 +1835,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A2" s="9" t="s">
         <v>66</v>
       </c>
@@ -1848,7 +1848,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A3" s="10" t="s">
         <v>89</v>
       </c>
@@ -1861,7 +1861,7 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A4" s="9" t="s">
         <v>90</v>
       </c>
@@ -1874,7 +1874,7 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A5" s="10" t="s">
         <v>74</v>
       </c>
@@ -1896,7 +1896,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A6" s="9" t="s">
         <v>97</v>
       </c>
@@ -1912,7 +1912,7 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A7" s="10" t="s">
         <v>100</v>
       </c>
@@ -1947,7 +1947,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A8" s="9" t="s">
         <v>95</v>
       </c>
@@ -1960,7 +1960,7 @@
       <c r="P8" s="1"/>
       <c r="Q8" s="1"/>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -1971,7 +1971,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>124</v>
       </c>
@@ -1982,12 +1982,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.35">
       <c r="A11" s="10"/>
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.35">
       <c r="Q12" s="1"/>
       <c r="R12" s="1"/>
     </row>
@@ -2021,21 +2021,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CABA7C5-6230-4207-9D35-0A95D86E66AC}">
   <dimension ref="A1:Q10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="20.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.08984375" bestFit="1" customWidth="1"/>
     <col min="4" max="6" width="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="25.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="9" max="10" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="13" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.6328125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="11.90625" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="13" width="18.36328125" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
-    <col min="15" max="17" width="21.5546875" bestFit="1" customWidth="1"/>
+    <col min="15" max="17" width="21.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2088,7 +2088,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
         <v>66</v>
       </c>
@@ -2113,7 +2113,7 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>89</v>
       </c>
@@ -2138,7 +2138,7 @@
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>90</v>
       </c>
@@ -2163,7 +2163,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>74</v>
       </c>
@@ -2202,7 +2202,7 @@
       </c>
       <c r="Q5" s="4"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>97</v>
       </c>
@@ -2235,7 +2235,7 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>100</v>
       </c>
@@ -2272,7 +2272,7 @@
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>95</v>
       </c>
@@ -2301,7 +2301,7 @@
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A9" s="10" t="s">
         <v>121</v>
       </c>
@@ -2318,7 +2318,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>124</v>
       </c>
@@ -2379,34 +2379,34 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C870BDA0-9E4C-481D-87BE-9D47789809C8}">
   <dimension ref="A1:AA10"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="5" width="25.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="27.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="25.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="36.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.5546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="23.109375" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="19.88671875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="10.5546875" customWidth="1"/>
-    <col min="17" max="17" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.88671875" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.88671875" customWidth="1"/>
-    <col min="21" max="21" width="12.88671875" customWidth="1"/>
-    <col min="22" max="23" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="35.33203125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.33203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="36.90625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="23.08984375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="19.90625" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.54296875" customWidth="1"/>
+    <col min="17" max="17" width="15.54296875" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.08984375" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.90625" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.90625" customWidth="1"/>
+    <col min="21" max="21" width="12.90625" customWidth="1"/>
+    <col min="22" max="23" width="17.90625" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="19.453125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="35.36328125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.36328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>26</v>
       </c>
@@ -2489,7 +2489,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>68</v>
       </c>
@@ -2548,7 +2548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>73</v>
       </c>
@@ -2604,7 +2604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>105</v>
       </c>
@@ -2660,7 +2660,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>113</v>
       </c>
@@ -2719,7 +2719,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>114</v>
       </c>
@@ -2757,7 +2757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>115</v>
       </c>
@@ -2816,7 +2816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>116</v>
       </c>
@@ -2854,7 +2854,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>117</v>
       </c>
@@ -2913,7 +2913,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -2976,22 +2976,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{981CFA5E-60F3-446F-A856-2FA65B76879A}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.88671875" customWidth="1"/>
-    <col min="8" max="8" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.08984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.54296875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.90625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.90625" customWidth="1"/>
+    <col min="8" max="8" width="12.90625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.109375" customWidth="1"/>
+    <col min="10" max="10" width="11.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.08984375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -3026,7 +3026,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>72</v>
       </c>
@@ -3052,7 +3052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>106</v>
       </c>
@@ -3107,122 +3107,122 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DC79B9-9C58-497E-9FD8-D3F2239E9BDC}">
   <dimension ref="A1:A23"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.90625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>104</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>125</v>
       </c>

</xml_diff>